<commit_message>
feat: add seed script and assessed sample data
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="127">
   <si>
     <t>lead_id</t>
   </si>
@@ -265,9 +265,6 @@
     <t>+91 00000 00013</t>
   </si>
   <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
     <t>L014</t>
   </si>
   <si>
@@ -305,9 +302,6 @@
   </si>
   <si>
     <t>+91 00000 00016</t>
-  </si>
-  <si>
-    <t>2026-10-18</t>
   </si>
   <si>
     <t>L017</t>
@@ -1135,7 +1129,7 @@
         <v>41</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="G14" t="s">
         <v>28</v>
@@ -1146,22 +1140,22 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" t="s">
         <v>85</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>86</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>87</v>
-      </c>
-      <c r="D15" t="s">
-        <v>88</v>
       </c>
       <c r="E15" t="s">
         <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="G15" t="s">
         <v>35</v>
@@ -1172,22 +1166,22 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" t="s">
         <v>89</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>90</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>91</v>
-      </c>
-      <c r="D16" t="s">
-        <v>92</v>
       </c>
       <c r="E16" t="s">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
         <v>43</v>
@@ -1198,22 +1192,22 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" t="s">
         <v>94</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>96</v>
-      </c>
-      <c r="D17" t="s">
-        <v>97</v>
       </c>
       <c r="E17" t="s">
         <v>41</v>
       </c>
       <c r="F17" t="s">
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="G17" t="s">
         <v>14</v>
@@ -1224,22 +1218,22 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" t="s">
         <v>99</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>100</v>
-      </c>
-      <c r="C18" t="s">
-        <v>101</v>
-      </c>
-      <c r="D18" t="s">
-        <v>102</v>
       </c>
       <c r="E18" t="s">
         <v>12</v>
       </c>
       <c r="F18" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G18" t="s">
         <v>21</v>
@@ -1250,22 +1244,22 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" t="s">
         <v>104</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>105</v>
-      </c>
-      <c r="C19" t="s">
-        <v>106</v>
-      </c>
-      <c r="D19" t="s">
-        <v>107</v>
       </c>
       <c r="E19" t="s">
         <v>27</v>
       </c>
       <c r="F19" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G19" t="s">
         <v>28</v>
@@ -1276,22 +1270,22 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" t="s">
         <v>109</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>110</v>
-      </c>
-      <c r="C20" t="s">
-        <v>111</v>
-      </c>
-      <c r="D20" t="s">
-        <v>112</v>
       </c>
       <c r="E20" t="s">
         <v>34</v>
       </c>
       <c r="F20" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G20" t="s">
         <v>35</v>
@@ -1302,22 +1296,22 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" t="s">
         <v>114</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>115</v>
-      </c>
-      <c r="C21" t="s">
-        <v>116</v>
-      </c>
-      <c r="D21" t="s">
-        <v>117</v>
       </c>
       <c r="E21" t="s">
         <v>41</v>
       </c>
       <c r="F21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G21" t="s">
         <v>43</v>
@@ -1328,22 +1322,22 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" t="s">
         <v>119</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
         <v>120</v>
-      </c>
-      <c r="C22" t="s">
-        <v>121</v>
-      </c>
-      <c r="D22" t="s">
-        <v>122</v>
       </c>
       <c r="E22" t="s">
         <v>12</v>
       </c>
       <c r="F22" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G22" t="s">
         <v>14</v>
@@ -1354,22 +1348,22 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" t="s">
         <v>124</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>125</v>
-      </c>
-      <c r="C23" t="s">
-        <v>126</v>
-      </c>
-      <c r="D23" t="s">
-        <v>127</v>
       </c>
       <c r="E23" t="s">
         <v>78</v>
       </c>
       <c r="F23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G23" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
chore: move sample data to 29 Oct and reseed with Groq
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -52,246 +52,246 @@
     <t>Trade show</t>
   </si>
   <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>Amit Verma</t>
+  </si>
+  <si>
+    <t>carton sealer</t>
+  </si>
+  <si>
+    <t>L002</t>
+  </si>
+  <si>
+    <t>Kavita Joshi</t>
+  </si>
+  <si>
+    <t>Sundrop Dairy Products</t>
+  </si>
+  <si>
+    <t>+91 00000 00002</t>
+  </si>
+  <si>
+    <t>Referral</t>
+  </si>
+  <si>
+    <t>Neha Kapoor</t>
+  </si>
+  <si>
+    <t>case erector</t>
+  </si>
+  <si>
+    <t>L003</t>
+  </si>
+  <si>
+    <t>Manish Ahuja</t>
+  </si>
+  <si>
+    <t>Zestora Beverages</t>
+  </si>
+  <si>
+    <t>+91 00000 00003</t>
+  </si>
+  <si>
+    <t>WhatsApp</t>
+  </si>
+  <si>
+    <t>Rahul Mehta</t>
+  </si>
+  <si>
+    <t>shrink wrapper</t>
+  </si>
+  <si>
+    <t>L004</t>
+  </si>
+  <si>
+    <t>Pooja Bansal</t>
+  </si>
+  <si>
+    <t>Nimbus Pharma Labs</t>
+  </si>
+  <si>
+    <t>+91 00000 00004</t>
+  </si>
+  <si>
+    <t>Website form</t>
+  </si>
+  <si>
+    <t>Sana Sheikh</t>
+  </si>
+  <si>
+    <t>labelling machine</t>
+  </si>
+  <si>
+    <t>L005</t>
+  </si>
+  <si>
+    <t>Rohit Chandra</t>
+  </si>
+  <si>
+    <t>Veloura Spices</t>
+  </si>
+  <si>
+    <t>+91 00000 00005</t>
+  </si>
+  <si>
+    <t>IndiaMART</t>
+  </si>
+  <si>
+    <t>2026-10-26</t>
+  </si>
+  <si>
+    <t>Vikram Rao</t>
+  </si>
+  <si>
+    <t>strapping machine</t>
+  </si>
+  <si>
+    <t>L006</t>
+  </si>
+  <si>
+    <t>Anita Deshpande</t>
+  </si>
+  <si>
+    <t>Cartly Online Retail</t>
+  </si>
+  <si>
+    <t>+91 00000 00006</t>
+  </si>
+  <si>
+    <t>L007</t>
+  </si>
+  <si>
+    <t>Sameer Qureshi</t>
+  </si>
+  <si>
+    <t>Aaromax Foods</t>
+  </si>
+  <si>
+    <t>+91 00000 00007</t>
+  </si>
+  <si>
     <t>2026-10-28</t>
   </si>
   <si>
-    <t>Amit Verma</t>
-  </si>
-  <si>
-    <t>carton sealer</t>
-  </si>
-  <si>
-    <t>L002</t>
-  </si>
-  <si>
-    <t>Kavita Joshi</t>
-  </si>
-  <si>
-    <t>Sundrop Dairy Products</t>
-  </si>
-  <si>
-    <t>+91 00000 00002</t>
-  </si>
-  <si>
-    <t>Referral</t>
-  </si>
-  <si>
-    <t>Neha Kapoor</t>
-  </si>
-  <si>
-    <t>case erector</t>
-  </si>
-  <si>
-    <t>L003</t>
-  </si>
-  <si>
-    <t>Manish Ahuja</t>
-  </si>
-  <si>
-    <t>Zestora Beverages</t>
-  </si>
-  <si>
-    <t>+91 00000 00003</t>
-  </si>
-  <si>
-    <t>WhatsApp</t>
-  </si>
-  <si>
-    <t>Rahul Mehta</t>
-  </si>
-  <si>
-    <t>shrink wrapper</t>
-  </si>
-  <si>
-    <t>L004</t>
-  </si>
-  <si>
-    <t>Pooja Bansal</t>
-  </si>
-  <si>
-    <t>Nimbus Pharma Labs</t>
-  </si>
-  <si>
-    <t>+91 00000 00004</t>
-  </si>
-  <si>
-    <t>Website form</t>
-  </si>
-  <si>
-    <t>Sana Sheikh</t>
-  </si>
-  <si>
-    <t>labelling machine</t>
-  </si>
-  <si>
-    <t>L005</t>
-  </si>
-  <si>
-    <t>Rohit Chandra</t>
-  </si>
-  <si>
-    <t>Veloura Spices</t>
-  </si>
-  <si>
-    <t>+91 00000 00005</t>
-  </si>
-  <si>
-    <t>IndiaMART</t>
+    <t>form-fill-seal</t>
+  </si>
+  <si>
+    <t>L008</t>
+  </si>
+  <si>
+    <t>Tanvi Kulkarni</t>
+  </si>
+  <si>
+    <t>Boltwave E-commerce</t>
+  </si>
+  <si>
+    <t>+91 00000 00008</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>L009</t>
+  </si>
+  <si>
+    <t>Farhan Ansari</t>
+  </si>
+  <si>
+    <t>Medora Healthcare</t>
+  </si>
+  <si>
+    <t>+91 00000 00009</t>
   </si>
   <si>
     <t>2026-10-25</t>
   </si>
   <si>
-    <t>Vikram Rao</t>
-  </si>
-  <si>
-    <t>strapping machine</t>
-  </si>
-  <si>
-    <t>L006</t>
-  </si>
-  <si>
-    <t>Anita Deshpande</t>
-  </si>
-  <si>
-    <t>Cartly Online Retail</t>
-  </si>
-  <si>
-    <t>+91 00000 00006</t>
-  </si>
-  <si>
-    <t>L007</t>
-  </si>
-  <si>
-    <t>Sameer Qureshi</t>
-  </si>
-  <si>
-    <t>Aaromax Foods</t>
-  </si>
-  <si>
-    <t>+91 00000 00007</t>
-  </si>
-  <si>
-    <t>2026-10-27</t>
-  </si>
-  <si>
-    <t>form-fill-seal</t>
-  </si>
-  <si>
-    <t>L008</t>
-  </si>
-  <si>
-    <t>Tanvi Kulkarni</t>
-  </si>
-  <si>
-    <t>Boltwave E-commerce</t>
-  </si>
-  <si>
-    <t>+91 00000 00008</t>
-  </si>
-  <si>
-    <t>2026-10-26</t>
-  </si>
-  <si>
-    <t>L009</t>
-  </si>
-  <si>
-    <t>Farhan Ansari</t>
-  </si>
-  <si>
-    <t>Medora Healthcare</t>
-  </si>
-  <si>
-    <t>+91 00000 00009</t>
+    <t>L010</t>
+  </si>
+  <si>
+    <t>Gaurav Pillai</t>
+  </si>
+  <si>
+    <t>Dalmera Dairy</t>
+  </si>
+  <si>
+    <t>+91 00000 00010</t>
+  </si>
+  <si>
+    <t>L011</t>
+  </si>
+  <si>
+    <t>Ritu Saxena</t>
+  </si>
+  <si>
+    <t>Crispo Namkeen</t>
+  </si>
+  <si>
+    <t>+91 00000 00011</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>L012</t>
+  </si>
+  <si>
+    <t>Harsh Vora</t>
+  </si>
+  <si>
+    <t>Lumina Nutraceuticals</t>
+  </si>
+  <si>
+    <t>+91 00000 00012</t>
+  </si>
+  <si>
+    <t>Cold call</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>L013</t>
+  </si>
+  <si>
+    <t>Deepak Naidu</t>
+  </si>
+  <si>
+    <t>Freshgrain Foods</t>
+  </si>
+  <si>
+    <t>+91 00000 00013</t>
+  </si>
+  <si>
+    <t>L014</t>
+  </si>
+  <si>
+    <t>Shalini Menon</t>
+  </si>
+  <si>
+    <t>Orbit Parcel Co</t>
+  </si>
+  <si>
+    <t>+91 00000 00014</t>
+  </si>
+  <si>
+    <t>L015</t>
+  </si>
+  <si>
+    <t>Arjun Bhatt</t>
+  </si>
+  <si>
+    <t>Gulmohar Frozen Foods</t>
+  </si>
+  <si>
+    <t>+91 00000 00015</t>
   </si>
   <si>
     <t>2026-10-24</t>
   </si>
   <si>
-    <t>L010</t>
-  </si>
-  <si>
-    <t>Gaurav Pillai</t>
-  </si>
-  <si>
-    <t>Dalmera Dairy</t>
-  </si>
-  <si>
-    <t>+91 00000 00010</t>
-  </si>
-  <si>
-    <t>L011</t>
-  </si>
-  <si>
-    <t>Ritu Saxena</t>
-  </si>
-  <si>
-    <t>Crispo Namkeen</t>
-  </si>
-  <si>
-    <t>+91 00000 00011</t>
-  </si>
-  <si>
-    <t>2026-10-20</t>
-  </si>
-  <si>
-    <t>L012</t>
-  </si>
-  <si>
-    <t>Harsh Vora</t>
-  </si>
-  <si>
-    <t>Lumina Nutraceuticals</t>
-  </si>
-  <si>
-    <t>+91 00000 00012</t>
-  </si>
-  <si>
-    <t>Cold call</t>
-  </si>
-  <si>
-    <t>2026-10-22</t>
-  </si>
-  <si>
-    <t>L013</t>
-  </si>
-  <si>
-    <t>Deepak Naidu</t>
-  </si>
-  <si>
-    <t>Freshgrain Foods</t>
-  </si>
-  <si>
-    <t>+91 00000 00013</t>
-  </si>
-  <si>
-    <t>L014</t>
-  </si>
-  <si>
-    <t>Shalini Menon</t>
-  </si>
-  <si>
-    <t>Orbit Parcel Co</t>
-  </si>
-  <si>
-    <t>+91 00000 00014</t>
-  </si>
-  <si>
-    <t>L015</t>
-  </si>
-  <si>
-    <t>Arjun Bhatt</t>
-  </si>
-  <si>
-    <t>Gulmohar Frozen Foods</t>
-  </si>
-  <si>
-    <t>+91 00000 00015</t>
-  </si>
-  <si>
-    <t>2026-10-23</t>
-  </si>
-  <si>
     <t>L016</t>
   </si>
   <si>
@@ -316,7 +316,7 @@
     <t>+91 00000 00017</t>
   </si>
   <si>
-    <t>2026-10-09</t>
+    <t>2026-10-10</t>
   </si>
   <si>
     <t>L018</t>
@@ -331,24 +331,24 @@
     <t>+91 00000 00018</t>
   </si>
   <si>
+    <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>L019</t>
+  </si>
+  <si>
+    <t>Sanjay Khanna</t>
+  </si>
+  <si>
+    <t>Healwell Pharma</t>
+  </si>
+  <si>
+    <t>+91 00000 00019</t>
+  </si>
+  <si>
     <t>2026-10-14</t>
   </si>
   <si>
-    <t>L019</t>
-  </si>
-  <si>
-    <t>Sanjay Khanna</t>
-  </si>
-  <si>
-    <t>Healwell Pharma</t>
-  </si>
-  <si>
-    <t>+91 00000 00019</t>
-  </si>
-  <si>
-    <t>2026-10-13</t>
-  </si>
-  <si>
     <t>L020</t>
   </si>
   <si>
@@ -361,7 +361,7 @@
     <t>+91 00000 00020</t>
   </si>
   <si>
-    <t>2026-10-03</t>
+    <t>2026-10-04</t>
   </si>
   <si>
     <t>L021</t>
@@ -376,7 +376,7 @@
     <t>+91 00000 00021</t>
   </si>
   <si>
-    <t>2026-09-20</t>
+    <t>2026-09-21</t>
   </si>
   <si>
     <t>L022</t>
@@ -391,7 +391,7 @@
     <t>+91 00000 00022</t>
   </si>
   <si>
-    <t>2026-09-30</t>
+    <t>2026-10-01</t>
   </si>
 </sst>
 </file>

</xml_diff>